<commit_message>
Fix capstone company size labels
</commit_message>
<xml_diff>
--- a/tasks/Data Analytics Capstone Project/outputs/google_sheets_dashboard/osmi_mental_health_google_sheets_dashboard.xlsx
+++ b/tasks/Data Analytics Capstone Project/outputs/google_sheets_dashboard/osmi_mental_health_google_sheets_dashboard.xlsx
@@ -379,7 +379,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5143500" cy="3057525"/>
+    <ext cx="5143500" cy="3305175"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -1101,7 +1101,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>These supporting visuals are included in the written report and kept here for dashboard audit/review.</t>
+          <t>Supporting visuals used in the written report and dashboard audit.</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>no_employees</t>
+          <t>company_size</t>
         </is>
       </c>
       <c r="B27" s="13" t="inlineStr">
@@ -1578,7 +1578,7 @@
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>1-5</t>
+          <t>1 to 5</t>
         </is>
       </c>
       <c r="B28" s="14" t="n">
@@ -1597,26 +1597,26 @@
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>100-500</t>
+          <t>6 to 25</t>
         </is>
       </c>
       <c r="B29" s="14" t="n">
-        <v>176</v>
+        <v>290</v>
       </c>
       <c r="C29" s="14" t="n">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="D29" s="14" t="n">
-        <v>0.5397727272727273</v>
+        <v>0.4413793103448276</v>
       </c>
       <c r="E29" s="14" t="n">
-        <v>54</v>
+        <v>44.1</v>
       </c>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>26-100</t>
+          <t>26 to 100</t>
         </is>
       </c>
       <c r="B30" s="14" t="n">
@@ -1635,26 +1635,26 @@
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>More than 1000</t>
+          <t>100 to 500</t>
         </is>
       </c>
       <c r="B31" s="14" t="n">
-        <v>282</v>
+        <v>176</v>
       </c>
       <c r="C31" s="14" t="n">
-        <v>146</v>
+        <v>95</v>
       </c>
       <c r="D31" s="14" t="n">
-        <v>0.5177304964539007</v>
+        <v>0.5397727272727273</v>
       </c>
       <c r="E31" s="14" t="n">
-        <v>51.8</v>
+        <v>54</v>
       </c>
     </row>
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>500-1000</t>
+          <t>500 to 1000</t>
         </is>
       </c>
       <c r="B32" s="14" t="n">
@@ -1673,20 +1673,20 @@
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>6-25</t>
+          <t>More than 1000</t>
         </is>
       </c>
       <c r="B33" s="14" t="n">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="C33" s="14" t="n">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="D33" s="14" t="n">
-        <v>0.4413793103448276</v>
+        <v>0.5177304964539007</v>
       </c>
       <c r="E33" s="14" t="n">
-        <v>44.1</v>
+        <v>51.8</v>
       </c>
     </row>
     <row r="34" ht="24" customHeight="1"/>
@@ -2260,12 +2260,12 @@
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>Difference in discussion_comfort_score across no_employees</t>
+          <t>Difference in discussion_comfort_score across company_size_label</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>no_employees</t>
+          <t>company_size_label</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -2301,12 +2301,12 @@
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>Difference in leave_difficulty_score across no_employees</t>
+          <t>Difference in leave_difficulty_score across company_size_label</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>no_employees</t>
+          <t>company_size_label</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>categorical__no_employees_500-1000</t>
+          <t>categorical__company_size_500 to 1000</t>
         </is>
       </c>
       <c r="B23" s="14" t="n">

</xml_diff>